<commit_message>
Replace Social Studies test scores file and update Science test scores file
</commit_message>
<xml_diff>
--- a/Science_Test_Scores.xlsx
+++ b/Science_Test_Scores.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
           <t>Test_1(%)</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Test_2(%)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -457,6 +462,9 @@
       <c r="C2" t="n">
         <v>42.86</v>
       </c>
+      <c r="D2" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -470,6 +478,9 @@
       <c r="C3" t="n">
         <v>41.43</v>
       </c>
+      <c r="D3" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -483,6 +494,9 @@
       <c r="C4" t="n">
         <v>62.86</v>
       </c>
+      <c r="D4" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -496,6 +510,9 @@
       <c r="C5" t="n">
         <v>48.57</v>
       </c>
+      <c r="D5" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -509,6 +526,9 @@
       <c r="C6" t="n">
         <v>38.57</v>
       </c>
+      <c r="D6" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -521,6 +541,9 @@
       </c>
       <c r="C7" t="n">
         <v>38.57</v>
+      </c>
+      <c r="D7" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>